<commit_message>
feat: add course registration limit and auto-assignment logic
- Implemented `getRegistrationLimit` function to determine maximum allowed course registration based on GPA.
- Added `autoAssignEligibleCourses` function to automatically assign courses for students based on academic priorities.
- Enhanced `excelProcessor` to include new registration workbook generation functions.
- Created `regFormGenerator` service to handle registration form Excel workbook generation with student details and course assignments.
- Introduced `rosterParser` for parsing student roster Excel files, including dynamic header detection for IDs and names.
</commit_message>
<xml_diff>
--- a/public/reg.xlsx
+++ b/public/reg.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mazenelnahla/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mazenelnahla/Desktop/Projects/React Projects/degree/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{953D80BD-7B5C-B34C-9A01-F70AE9B977FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A09D760D-A452-134E-80F1-0DB5FE64A9DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="1200" windowWidth="28040" windowHeight="17180" xr2:uid="{939E2F63-55F2-5040-8EF3-9B8F382D797F}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="28">
   <si>
     <t>East Port Said National University</t>
   </si>
@@ -108,22 +108,7 @@
     <t>Course Title</t>
   </si>
   <si>
-    <t>Second level Courses</t>
-  </si>
-  <si>
-    <t>EPM 213: Electronics &amp; Digital Circuits</t>
-  </si>
-  <si>
-    <t>CCE 112: Computer Programming 2</t>
-  </si>
-  <si>
-    <t>CCE 211: Data Structures &amp; Algorithms</t>
-  </si>
-  <si>
     <t>Other Courses</t>
-  </si>
-  <si>
-    <t>EPM 116: Electrical Circuits &amp; Measurements 1</t>
   </si>
   <si>
     <t>Total Credit Hour Registered</t>
@@ -227,7 +212,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -356,75 +341,18 @@
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" readingOrder="1"/>
@@ -445,12 +373,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -470,12 +392,6 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -490,12 +406,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1" readingOrder="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
@@ -509,17 +422,16 @@
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
@@ -649,297 +561,6 @@
         <row r="8">
           <cell r="G8">
             <v>3</v>
-          </cell>
-          <cell r="H8" t="str">
-            <v>BSC 011: Mathematics I</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="G9">
-            <v>3</v>
-          </cell>
-          <cell r="H9" t="str">
-            <v>BSC 031: Physics I</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="G10">
-            <v>3</v>
-          </cell>
-          <cell r="H10" t="str">
-            <v>BSC 021: Mechanics I</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="G11">
-            <v>3</v>
-          </cell>
-          <cell r="H11" t="str">
-            <v>BSC 041: Chemical Engineering</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="G12">
-            <v>3</v>
-          </cell>
-          <cell r="H12" t="str">
-            <v>PRD 031: Engineering Drawing and Projection</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="G13">
-            <v>1</v>
-          </cell>
-          <cell r="H13" t="str">
-            <v>GUR 0C1: Law and Human Rights</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="G14">
-            <v>3</v>
-          </cell>
-          <cell r="H14" t="str">
-            <v>BSC 012: Mathematics II</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="G15">
-            <v>3</v>
-          </cell>
-          <cell r="H15" t="str">
-            <v>BSC 032: Physics II</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="G16">
-            <v>3</v>
-          </cell>
-          <cell r="H16" t="str">
-            <v>BSC 022: Mechanics II</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="G17">
-            <v>3</v>
-          </cell>
-          <cell r="H17" t="str">
-            <v>PRD 041: Production Technology</v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="G18">
-            <v>3</v>
-          </cell>
-          <cell r="H18" t="str">
-            <v>CCE 031: Introduction to Computer Science</v>
-          </cell>
-        </row>
-        <row r="19">
-          <cell r="G19">
-            <v>2</v>
-          </cell>
-          <cell r="H19" t="str">
-            <v>GUR 0C2: English Language 1</v>
-          </cell>
-        </row>
-        <row r="20">
-          <cell r="G20">
-            <v>3</v>
-          </cell>
-          <cell r="H20" t="str">
-            <v>EPM 113: Electromagnetic Fields</v>
-          </cell>
-        </row>
-        <row r="21">
-          <cell r="G21">
-            <v>3</v>
-          </cell>
-          <cell r="H21" t="str">
-            <v>EPM 116: Electrical Circuits &amp; Measurements 1</v>
-          </cell>
-        </row>
-        <row r="22">
-          <cell r="G22">
-            <v>3</v>
-          </cell>
-          <cell r="H22" t="str">
-            <v>CCE 141: Logic Design 1</v>
-          </cell>
-        </row>
-        <row r="23">
-          <cell r="G23">
-            <v>3</v>
-          </cell>
-          <cell r="H23" t="str">
-            <v>CCE 111: Computer Programming 1</v>
-          </cell>
-        </row>
-        <row r="24">
-          <cell r="G24">
-            <v>3</v>
-          </cell>
-          <cell r="H24" t="str">
-            <v>BSC 111: Mathematics III</v>
-          </cell>
-        </row>
-        <row r="25">
-          <cell r="G25">
-            <v>2</v>
-          </cell>
-          <cell r="H25" t="str">
-            <v>GUR 1C1: Computer Skills</v>
-          </cell>
-        </row>
-        <row r="26">
-          <cell r="G26">
-            <v>3</v>
-          </cell>
-          <cell r="H26" t="str">
-            <v>BSC 112: Statistics &amp; Numerical Analysis</v>
-          </cell>
-        </row>
-        <row r="27">
-          <cell r="G27">
-            <v>3</v>
-          </cell>
-          <cell r="H27" t="str">
-            <v>EPM 117: Electrical Circuits &amp; Measurements 2</v>
-          </cell>
-        </row>
-        <row r="28">
-          <cell r="G28">
-            <v>3</v>
-          </cell>
-          <cell r="H28" t="str">
-            <v>CCE 142: Logic Design 2</v>
-          </cell>
-        </row>
-        <row r="29">
-          <cell r="G29">
-            <v>3</v>
-          </cell>
-          <cell r="H29" t="str">
-            <v>CCE 112: Computer Programming 2</v>
-          </cell>
-        </row>
-        <row r="30">
-          <cell r="G30">
-            <v>3</v>
-          </cell>
-          <cell r="H30" t="str">
-            <v>CCE 131: Mathematics for Machine Learning</v>
-          </cell>
-        </row>
-        <row r="31">
-          <cell r="G31">
-            <v>2</v>
-          </cell>
-          <cell r="H31" t="str">
-            <v>GUR 1C2: University Requirement (4)</v>
-          </cell>
-        </row>
-        <row r="32">
-          <cell r="G32">
-            <v>3</v>
-          </cell>
-          <cell r="H32" t="str">
-            <v>EPM 213: Electronics &amp; Digital Circuits</v>
-          </cell>
-        </row>
-        <row r="33">
-          <cell r="G33">
-            <v>3</v>
-          </cell>
-          <cell r="H33" t="str">
-            <v>CCE 221: Control Systems Engineering 1</v>
-          </cell>
-        </row>
-        <row r="34">
-          <cell r="G34">
-            <v>3</v>
-          </cell>
-          <cell r="H34" t="str">
-            <v>CCE 231: Machine Learning 1</v>
-          </cell>
-        </row>
-        <row r="35">
-          <cell r="G35">
-            <v>3</v>
-          </cell>
-          <cell r="H35" t="str">
-            <v>CCE 211: Data Structures &amp; Algorithms</v>
-          </cell>
-        </row>
-        <row r="36">
-          <cell r="G36">
-            <v>2</v>
-          </cell>
-          <cell r="H36" t="str">
-            <v>GUR 2C1: Research and Analysis Skills</v>
-          </cell>
-        </row>
-        <row r="37">
-          <cell r="G37">
-            <v>2</v>
-          </cell>
-          <cell r="H37" t="str">
-            <v>GUR 2E1: Presentation Skills</v>
-          </cell>
-        </row>
-        <row r="38">
-          <cell r="G38">
-            <v>1</v>
-          </cell>
-          <cell r="H38" t="str">
-            <v>GFR 2XX: Summer Training (1)</v>
-          </cell>
-        </row>
-        <row r="39">
-          <cell r="G39">
-            <v>3</v>
-          </cell>
-          <cell r="H39" t="str">
-            <v>CCE 241: Computer Architecture &amp; Organization</v>
-          </cell>
-        </row>
-        <row r="40">
-          <cell r="G40">
-            <v>3</v>
-          </cell>
-          <cell r="H40" t="str">
-            <v>CCE 222: Control Systems Engineering 2</v>
-          </cell>
-        </row>
-        <row r="41">
-          <cell r="G41">
-            <v>3</v>
-          </cell>
-          <cell r="H41" t="str">
-            <v>CCE 232: Machine Learning 2</v>
-          </cell>
-        </row>
-        <row r="42">
-          <cell r="G42">
-            <v>3</v>
-          </cell>
-          <cell r="H42" t="str">
-            <v>CCE 242: Digital Signal Processing</v>
-          </cell>
-        </row>
-        <row r="43">
-          <cell r="G43">
-            <v>3</v>
-          </cell>
-          <cell r="H43" t="str">
-            <v>CCE 212: Database Systems</v>
-          </cell>
-        </row>
-        <row r="44">
-          <cell r="G44">
-            <v>2</v>
-          </cell>
-          <cell r="H44" t="str">
-            <v>GUR 2E2: Mangement and Marketing</v>
           </cell>
         </row>
       </sheetData>
@@ -1728,7 +1349,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFDBFC1B-334F-4E4E-9066-E791E185699D}">
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="11.1640625" bestFit="1" customWidth="1"/>
@@ -1750,56 +1371,56 @@
     <row r="2" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="2"/>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="2"/>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
       <c r="G3" s="2"/>
     </row>
     <row r="4" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="2"/>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="20"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
       <c r="G4" s="2"/>
     </row>
     <row r="5" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="2"/>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="20"/>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16"/>
       <c r="G5" s="2"/>
     </row>
     <row r="6" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="2"/>
-      <c r="C6" s="21" t="s">
+      <c r="C6" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="20"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
       <c r="G6" s="2"/>
     </row>
     <row r="7" spans="1:7" ht="20" thickBot="1" x14ac:dyDescent="0.3">
@@ -1819,11 +1440,11 @@
       <c r="C8" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D8" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="E8" s="12"/>
-      <c r="F8" s="13"/>
+      <c r="D8" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" s="10"/>
+      <c r="F8" s="11"/>
       <c r="G8" s="3" t="s">
         <v>7</v>
       </c>
@@ -1837,9 +1458,9 @@
       <c r="C9" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D9" s="29"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="13"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="11"/>
       <c r="G9" s="3" t="s">
         <v>9</v>
       </c>
@@ -1863,14 +1484,14 @@
     </row>
     <row r="11" spans="1:7" ht="20" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
-      <c r="B11" s="30"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="31" t="s">
+      <c r="B11" s="23"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="G11" s="13"/>
+      <c r="G11" s="11"/>
     </row>
     <row r="12" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
@@ -1883,15 +1504,15 @@
     </row>
     <row r="13" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A13" s="1"/>
-      <c r="B13" s="32" t="s">
+      <c r="B13" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="33"/>
-      <c r="D13" s="23"/>
-      <c r="E13" s="32" t="s">
+      <c r="C13" s="26"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="F13" s="23"/>
+      <c r="F13" s="19"/>
       <c r="G13" s="5"/>
     </row>
     <row r="14" spans="1:7" ht="20" x14ac:dyDescent="0.2">
@@ -1899,172 +1520,149 @@
       <c r="B14" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="22" t="s">
+      <c r="C14" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="D14" s="23"/>
+      <c r="D14" s="19"/>
       <c r="E14" s="6" t="s">
         <v>19</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="G14" s="24" t="s">
-        <v>21</v>
-      </c>
+      <c r="G14" s="20"/>
     </row>
     <row r="15" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A15" s="1"/>
-      <c r="B15" s="7">
-        <f t="array" ref="B15">IFERROR(INDEX('[1]AI Subjects'!$G$8:$G$44, MATCH(C15, '[1]AI Subjects'!$H$8:$H$44, 0)), "")</f>
-        <v>3</v>
-      </c>
-      <c r="C15" s="27" t="s">
-        <v>22</v>
-      </c>
-      <c r="D15" s="28"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="30"/>
       <c r="E15" s="6"/>
-      <c r="F15" s="8"/>
-      <c r="G15" s="25"/>
-    </row>
-    <row r="16" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="F15" s="6"/>
+      <c r="G15" s="21"/>
+    </row>
+    <row r="16" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A16" s="1"/>
-      <c r="B16" s="7">
-        <f t="array" ref="B16">IFERROR(INDEX('[1]AI Subjects'!$G$8:$G$44, MATCH(C16, '[1]AI Subjects'!$H$8:$H$44, 0)), "")</f>
-        <v>3</v>
-      </c>
-      <c r="C16" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="D16" s="18"/>
-      <c r="E16" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="F16" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="G16" s="26"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="30"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="21"/>
     </row>
     <row r="17" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
-      <c r="B17" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="C17" s="15"/>
-      <c r="D17" s="15"/>
-      <c r="E17" s="15"/>
-      <c r="F17" s="15"/>
-      <c r="G17" s="16"/>
-    </row>
-    <row r="18" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="B17" s="6"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="30"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="21"/>
+    </row>
+    <row r="18" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A18" s="1"/>
-      <c r="B18" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C18" s="22" t="s">
-        <v>18</v>
-      </c>
-      <c r="D18" s="23"/>
-      <c r="E18" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F18" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="G18" s="23"/>
+      <c r="B18" s="6"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="30"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="21"/>
     </row>
     <row r="19" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A19" s="1"/>
-      <c r="B19" s="7">
-        <f t="array" ref="B19">IFERROR(INDEX('[1]AI Subjects'!$G$8:$G$44, MATCH(C19, '[1]AI Subjects'!$H$8:$H$44, 0)), "")</f>
-        <v>3</v>
-      </c>
-      <c r="C19" s="17" t="s">
-        <v>26</v>
-      </c>
-      <c r="D19" s="23"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="30"/>
       <c r="E19" s="6"/>
-      <c r="F19" s="34"/>
-      <c r="G19" s="23"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="21"/>
     </row>
     <row r="20" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>
-      <c r="B20" s="7"/>
-      <c r="C20" s="27"/>
-      <c r="D20" s="28"/>
+      <c r="B20" s="6"/>
+      <c r="C20" s="18"/>
+      <c r="D20" s="30"/>
       <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="21"/>
     </row>
     <row r="21" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A21" s="1"/>
-      <c r="B21" s="7"/>
-      <c r="C21" s="35"/>
-      <c r="D21" s="28"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="34"/>
-      <c r="G21" s="23"/>
-    </row>
-    <row r="22" spans="1:7" ht="19" x14ac:dyDescent="0.2">
+      <c r="B21" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="13"/>
+      <c r="F21" s="13"/>
+      <c r="G21" s="14"/>
+    </row>
+    <row r="22" spans="1:7" ht="20" x14ac:dyDescent="0.2">
       <c r="A22" s="1"/>
-      <c r="B22" s="7"/>
-      <c r="C22" s="36"/>
-      <c r="D22" s="37"/>
-      <c r="E22" s="6"/>
-      <c r="F22" s="34"/>
-      <c r="G22" s="23"/>
+      <c r="B22" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C22" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D22" s="19"/>
+      <c r="E22" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F22" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G22" s="19"/>
     </row>
     <row r="23" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A23" s="1"/>
       <c r="B23" s="7"/>
-      <c r="C23" s="17"/>
-      <c r="D23" s="23"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="19"/>
       <c r="E23" s="6"/>
-      <c r="F23" s="34"/>
-      <c r="G23" s="23"/>
+      <c r="F23" s="28"/>
+      <c r="G23" s="19"/>
     </row>
     <row r="24" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A24" s="1"/>
-      <c r="B24" s="5">
-        <f>SUM(B15:B16,B19:B23)</f>
-        <v>9</v>
-      </c>
-      <c r="C24" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="D24" s="33"/>
-      <c r="E24" s="33"/>
-      <c r="F24" s="33"/>
-      <c r="G24" s="23"/>
-    </row>
-    <row r="25" spans="1:7" ht="19" x14ac:dyDescent="0.25">
+      <c r="B24" s="7"/>
+      <c r="C24" s="27"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="28"/>
+      <c r="G24" s="19"/>
+    </row>
+    <row r="25" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A25" s="1"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-    </row>
-    <row r="26" spans="1:7" ht="20" x14ac:dyDescent="0.25">
+      <c r="B25" s="7"/>
+      <c r="C25" s="27"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="6"/>
+      <c r="F25" s="28"/>
+      <c r="G25" s="19"/>
+    </row>
+    <row r="26" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A26" s="1"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="10"/>
-      <c r="D26" s="38" t="s">
-        <v>28</v>
-      </c>
-      <c r="E26" s="20"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="10" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="19" x14ac:dyDescent="0.25">
+      <c r="B26" s="7"/>
+      <c r="C26" s="27"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="28"/>
+      <c r="G26" s="19"/>
+    </row>
+    <row r="27" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A27" s="1"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="38"/>
-      <c r="E27" s="20"/>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
+      <c r="B27" s="5">
+        <f>SUM(B15:B20,B23:B26)</f>
+        <v>0</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D27" s="26"/>
+      <c r="E27" s="26"/>
+      <c r="F27" s="26"/>
+      <c r="G27" s="19"/>
     </row>
     <row r="28" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
@@ -2075,57 +1673,91 @@
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
     </row>
-    <row r="29" spans="1:7" ht="19" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" ht="20" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
-      <c r="B29" s="38" t="s">
-        <v>30</v>
-      </c>
-      <c r="C29" s="20"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
+      <c r="B29" s="2"/>
+      <c r="C29" s="8"/>
+      <c r="D29" s="29" t="s">
+        <v>23</v>
+      </c>
+      <c r="E29" s="16"/>
       <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
+      <c r="G29" s="8" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="30" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
-      <c r="B30" s="38" t="s">
-        <v>31</v>
-      </c>
-      <c r="C30" s="20"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
+      <c r="B30" s="2"/>
+      <c r="C30" s="2"/>
+      <c r="D30" s="29"/>
+      <c r="E30" s="16"/>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
     </row>
+    <row r="31" spans="1:7" ht="19" x14ac:dyDescent="0.25">
+      <c r="A31" s="1"/>
+      <c r="B31" s="2"/>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
+      <c r="E31" s="2"/>
+      <c r="F31" s="2"/>
+      <c r="G31" s="2"/>
+    </row>
+    <row r="32" spans="1:7" ht="19" x14ac:dyDescent="0.25">
+      <c r="A32" s="1"/>
+      <c r="B32" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="C32" s="16"/>
+      <c r="D32" s="2"/>
+      <c r="E32" s="2"/>
+      <c r="F32" s="2"/>
+      <c r="G32" s="2"/>
+    </row>
+    <row r="33" spans="1:7" ht="19" x14ac:dyDescent="0.25">
+      <c r="A33" s="1"/>
+      <c r="B33" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="C33" s="16"/>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2"/>
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
+    </row>
   </sheetData>
-  <mergeCells count="32">
-    <mergeCell ref="C24:G24"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B30:C30"/>
+  <mergeCells count="35">
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="C27:G27"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="F22:G22"/>
     <mergeCell ref="C23:D23"/>
     <mergeCell ref="F23:G23"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="F24:G24"/>
     <mergeCell ref="D8:F8"/>
-    <mergeCell ref="B17:G17"/>
-    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="B21:G21"/>
     <mergeCell ref="C2:F2"/>
     <mergeCell ref="C3:F3"/>
     <mergeCell ref="C4:F4"/>
     <mergeCell ref="C5:F5"/>
     <mergeCell ref="C6:F6"/>
     <mergeCell ref="C14:D14"/>
-    <mergeCell ref="G14:G16"/>
-    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="G14:G20"/>
     <mergeCell ref="D9:F9"/>
     <mergeCell ref="B11:E11"/>
     <mergeCell ref="F11:G11"/>

</xml_diff>

<commit_message>
feat: add project backup/restore functionality and exported degree workbook parsing
</commit_message>
<xml_diff>
--- a/public/reg.xlsx
+++ b/public/reg.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mazenelnahla/Desktop/Projects/React Projects/degree/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A09D760D-A452-134E-80F1-0DB5FE64A9DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8839EAB4-6079-9944-98AB-9A8B24FED7D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="1200" windowWidth="28040" windowHeight="17180" xr2:uid="{939E2F63-55F2-5040-8EF3-9B8F382D797F}"/>
   </bookViews>
@@ -378,14 +378,32 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
@@ -395,14 +413,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1" readingOrder="1"/>
     </xf>
@@ -419,19 +432,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
@@ -456,9 +456,9 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>104775</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>209550</xdr:rowOff>
+      <xdr:colOff>15875</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="990600" cy="781050"/>
     <xdr:pic>
@@ -480,7 +480,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="15829429225" y="171450"/>
+          <a:off x="13528989325" y="298450"/>
           <a:ext cx="990600" cy="781050"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1371,56 +1371,56 @@
     <row r="2" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="2"/>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="2"/>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
       <c r="G3" s="2"/>
     </row>
     <row r="4" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="2"/>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="16"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
       <c r="G4" s="2"/>
     </row>
     <row r="5" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="2"/>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="16"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
       <c r="G5" s="2"/>
     </row>
     <row r="6" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="2"/>
-      <c r="C6" s="17" t="s">
+      <c r="C6" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="16"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="16"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
       <c r="G6" s="2"/>
     </row>
     <row r="7" spans="1:7" ht="20" thickBot="1" x14ac:dyDescent="0.3">
@@ -1440,11 +1440,11 @@
       <c r="C8" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="E8" s="10"/>
-      <c r="F8" s="11"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="20"/>
       <c r="G8" s="3" t="s">
         <v>7</v>
       </c>
@@ -1458,9 +1458,9 @@
       <c r="C9" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D9" s="22"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="11"/>
+      <c r="D9" s="27"/>
+      <c r="E9" s="19"/>
+      <c r="F9" s="20"/>
       <c r="G9" s="3" t="s">
         <v>9</v>
       </c>
@@ -1484,14 +1484,14 @@
     </row>
     <row r="11" spans="1:7" ht="20" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
-      <c r="B11" s="23"/>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="24" t="s">
+      <c r="B11" s="28"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="20"/>
+      <c r="F11" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="G11" s="11"/>
+      <c r="G11" s="20"/>
     </row>
     <row r="12" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
@@ -1504,15 +1504,15 @@
     </row>
     <row r="13" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A13" s="1"/>
-      <c r="B13" s="25" t="s">
+      <c r="B13" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="26"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="25" t="s">
+      <c r="C13" s="17"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="F13" s="19"/>
+      <c r="F13" s="14"/>
       <c r="G13" s="5"/>
     </row>
     <row r="14" spans="1:7" ht="20" x14ac:dyDescent="0.2">
@@ -1520,135 +1520,135 @@
       <c r="B14" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="18" t="s">
+      <c r="C14" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="D14" s="19"/>
+      <c r="D14" s="14"/>
       <c r="E14" s="6" t="s">
         <v>19</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="G14" s="20"/>
+      <c r="G14" s="25"/>
     </row>
     <row r="15" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A15" s="1"/>
       <c r="B15" s="6"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="30"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="12"/>
       <c r="E15" s="6"/>
       <c r="F15" s="6"/>
-      <c r="G15" s="21"/>
+      <c r="G15" s="26"/>
     </row>
     <row r="16" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A16" s="1"/>
       <c r="B16" s="6"/>
-      <c r="C16" s="18"/>
-      <c r="D16" s="30"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="12"/>
       <c r="E16" s="6"/>
       <c r="F16" s="6"/>
-      <c r="G16" s="21"/>
+      <c r="G16" s="26"/>
     </row>
     <row r="17" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
       <c r="B17" s="6"/>
-      <c r="C17" s="18"/>
-      <c r="D17" s="30"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="12"/>
       <c r="E17" s="6"/>
       <c r="F17" s="6"/>
-      <c r="G17" s="21"/>
+      <c r="G17" s="26"/>
     </row>
     <row r="18" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A18" s="1"/>
       <c r="B18" s="6"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="30"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="12"/>
       <c r="E18" s="6"/>
       <c r="F18" s="6"/>
-      <c r="G18" s="21"/>
+      <c r="G18" s="26"/>
     </row>
     <row r="19" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A19" s="1"/>
       <c r="B19" s="6"/>
-      <c r="C19" s="18"/>
-      <c r="D19" s="30"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="12"/>
       <c r="E19" s="6"/>
       <c r="F19" s="6"/>
-      <c r="G19" s="21"/>
+      <c r="G19" s="26"/>
     </row>
     <row r="20" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>
       <c r="B20" s="6"/>
-      <c r="C20" s="18"/>
-      <c r="D20" s="30"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="12"/>
       <c r="E20" s="6"/>
       <c r="F20" s="6"/>
-      <c r="G20" s="21"/>
+      <c r="G20" s="26"/>
     </row>
     <row r="21" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A21" s="1"/>
-      <c r="B21" s="12" t="s">
+      <c r="B21" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="13"/>
-      <c r="F21" s="13"/>
-      <c r="G21" s="14"/>
+      <c r="C21" s="21"/>
+      <c r="D21" s="21"/>
+      <c r="E21" s="21"/>
+      <c r="F21" s="21"/>
+      <c r="G21" s="22"/>
     </row>
     <row r="22" spans="1:7" ht="20" x14ac:dyDescent="0.2">
       <c r="A22" s="1"/>
       <c r="B22" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C22" s="18" t="s">
+      <c r="C22" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="D22" s="19"/>
+      <c r="D22" s="14"/>
       <c r="E22" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F22" s="18" t="s">
+      <c r="F22" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="G22" s="19"/>
+      <c r="G22" s="14"/>
     </row>
     <row r="23" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A23" s="1"/>
       <c r="B23" s="7"/>
-      <c r="C23" s="27"/>
-      <c r="D23" s="19"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="14"/>
       <c r="E23" s="6"/>
-      <c r="F23" s="28"/>
-      <c r="G23" s="19"/>
+      <c r="F23" s="15"/>
+      <c r="G23" s="14"/>
     </row>
     <row r="24" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A24" s="1"/>
       <c r="B24" s="7"/>
-      <c r="C24" s="27"/>
-      <c r="D24" s="19"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="14"/>
       <c r="E24" s="6"/>
-      <c r="F24" s="28"/>
-      <c r="G24" s="19"/>
+      <c r="F24" s="15"/>
+      <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A25" s="1"/>
       <c r="B25" s="7"/>
-      <c r="C25" s="27"/>
-      <c r="D25" s="19"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="14"/>
       <c r="E25" s="6"/>
-      <c r="F25" s="28"/>
-      <c r="G25" s="19"/>
+      <c r="F25" s="15"/>
+      <c r="G25" s="14"/>
     </row>
     <row r="26" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A26" s="1"/>
       <c r="B26" s="7"/>
-      <c r="C26" s="27"/>
-      <c r="D26" s="19"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="14"/>
       <c r="E26" s="6"/>
-      <c r="F26" s="28"/>
-      <c r="G26" s="19"/>
+      <c r="F26" s="15"/>
+      <c r="G26" s="14"/>
     </row>
     <row r="27" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A27" s="1"/>
@@ -1656,13 +1656,13 @@
         <f>SUM(B15:B20,B23:B26)</f>
         <v>0</v>
       </c>
-      <c r="C27" s="12" t="s">
+      <c r="C27" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="D27" s="26"/>
-      <c r="E27" s="26"/>
-      <c r="F27" s="26"/>
-      <c r="G27" s="19"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="14"/>
     </row>
     <row r="28" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
@@ -1677,10 +1677,10 @@
       <c r="A29" s="1"/>
       <c r="B29" s="2"/>
       <c r="C29" s="8"/>
-      <c r="D29" s="29" t="s">
+      <c r="D29" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E29" s="16"/>
+      <c r="E29" s="10"/>
       <c r="F29" s="2"/>
       <c r="G29" s="8" t="s">
         <v>24</v>
@@ -1690,8 +1690,8 @@
       <c r="A30" s="1"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
-      <c r="D30" s="29"/>
-      <c r="E30" s="16"/>
+      <c r="D30" s="9"/>
+      <c r="E30" s="10"/>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
     </row>
@@ -1706,10 +1706,10 @@
     </row>
     <row r="32" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
-      <c r="B32" s="29" t="s">
+      <c r="B32" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C32" s="16"/>
+      <c r="C32" s="10"/>
       <c r="D32" s="2"/>
       <c r="E32" s="2"/>
       <c r="F32" s="2"/>
@@ -1717,10 +1717,10 @@
     </row>
     <row r="33" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
-      <c r="B33" s="29" t="s">
+      <c r="B33" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="C33" s="16"/>
+      <c r="C33" s="10"/>
       <c r="D33" s="2"/>
       <c r="E33" s="2"/>
       <c r="F33" s="2"/>
@@ -1728,27 +1728,6 @@
     </row>
   </sheetData>
   <mergeCells count="35">
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="F26:G26"/>
-    <mergeCell ref="C27:G27"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="F23:G23"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="F24:G24"/>
     <mergeCell ref="D8:F8"/>
     <mergeCell ref="B21:G21"/>
     <mergeCell ref="C2:F2"/>
@@ -1763,6 +1742,27 @@
     <mergeCell ref="F11:G11"/>
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="E13:F13"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="C27:G27"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="F23:G23"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C25:D25"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
solved issues for ai program transcript reader
</commit_message>
<xml_diff>
--- a/public/reg.xlsx
+++ b/public/reg.xlsx
@@ -8,16 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mazenelnahla/Desktop/Projects/React Projects/degree/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8839EAB4-6079-9944-98AB-9A8B24FED7D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92530952-6AE8-ED46-8FEC-EE3FF8FD4B65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="1200" windowWidth="28040" windowHeight="17180" xr2:uid="{939E2F63-55F2-5040-8EF3-9B8F382D797F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId2"/>
-  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -42,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="29">
   <si>
     <t>East Port Said National University</t>
   </si>
@@ -127,6 +124,9 @@
   </si>
   <si>
     <t>name here</t>
+  </si>
+  <si>
+    <t/>
   </si>
 </sst>
 </file>
@@ -378,60 +378,60 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
@@ -530,506 +530,6 @@
     <xdr:clientData fLocksWithSheet="0"/>
   </xdr:oneCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-      <xxl21:relativeUrl r:id="rId3"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="AI Subjects"/>
-      <sheetName val="1st AI-Course Tree"/>
-      <sheetName val="1st AI-form"/>
-      <sheetName val="1st AI-Print"/>
-      <sheetName val="2nd AI-Course Tree"/>
-      <sheetName val="2nd AI-form"/>
-      <sheetName val="2nd AI-Print"/>
-      <sheetName val="3rd-Stu. Names"/>
-      <sheetName val="3rd AI-Course Tree"/>
-      <sheetName val="3rd AI-Form"/>
-      <sheetName val="ميكاترونيكس طباعة "/>
-      <sheetName val="تشييد ثالثة"/>
-      <sheetName val="CEP Subjects"/>
-      <sheetName val="SHEET#3CEP "/>
-      <sheetName val="3rd AI-Print"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0">
-        <row r="8">
-          <cell r="G8">
-            <v>3</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6">
-        <row r="9">
-          <cell r="D9">
-            <v>24130007</v>
-          </cell>
-          <cell r="E9" t="str">
-            <v>احمد اسامه عبد الرحمن ابراهيم حسن</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="D10">
-            <v>24130012</v>
-          </cell>
-          <cell r="E10" t="str">
-            <v>احمد سمير محمد السيد سعيد</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="D11">
-            <v>24130014</v>
-          </cell>
-          <cell r="E11" t="str">
-            <v>احمد طارق محمد حلمى محمد الروبى</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="D12">
-            <v>24130019</v>
-          </cell>
-          <cell r="E12" t="str">
-            <v>احمد عماد محمد جاد</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="D13">
-            <v>24130021</v>
-          </cell>
-          <cell r="E13" t="str">
-            <v>احمد محمود هانئ محمد فهمى</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="D14">
-            <v>24130030</v>
-          </cell>
-          <cell r="E14" t="str">
-            <v>المعتز بالله خالد رمضان طه محمد الكفراوي</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="D15">
-            <v>24130033</v>
-          </cell>
-          <cell r="E15" t="str">
-            <v>اواب عاطف مهدي محمد الجزار</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="D16">
-            <v>24130034</v>
-          </cell>
-          <cell r="E16" t="str">
-            <v>باسل السيد محمد احمد سليمان</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="D17">
-            <v>24130037</v>
-          </cell>
-          <cell r="E17" t="str">
-            <v>بسمله محمد احمد محمد المر</v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="D18">
-            <v>24130038</v>
-          </cell>
-          <cell r="E18" t="str">
-            <v>بسمه عبد الناصر عبد النعيم ابراهيم السيد</v>
-          </cell>
-        </row>
-        <row r="19">
-          <cell r="D19">
-            <v>24130041</v>
-          </cell>
-          <cell r="E19" t="str">
-            <v>جنا احمد عبدالحفيظ سليم</v>
-          </cell>
-        </row>
-        <row r="20">
-          <cell r="D20">
-            <v>24130042</v>
-          </cell>
-          <cell r="E20" t="str">
-            <v>جنه محمد السيد محمد الصاوى</v>
-          </cell>
-        </row>
-        <row r="21">
-          <cell r="D21">
-            <v>24130043</v>
-          </cell>
-          <cell r="E21" t="str">
-            <v>جنى عثمان احمد احمد يوسف فياض</v>
-          </cell>
-        </row>
-        <row r="22">
-          <cell r="D22">
-            <v>24130048</v>
-          </cell>
-          <cell r="E22" t="str">
-            <v>داليا ابراهيم علي ابراهيم مطراوي</v>
-          </cell>
-        </row>
-        <row r="23">
-          <cell r="D23">
-            <v>24130052</v>
-          </cell>
-          <cell r="E23" t="str">
-            <v>روان خالد عبد الواحد محمد عبد الواحد</v>
-          </cell>
-        </row>
-        <row r="24">
-          <cell r="D24">
-            <v>24130053</v>
-          </cell>
-          <cell r="E24" t="str">
-            <v>روان رضا موسى اسماعيل الجوهري</v>
-          </cell>
-        </row>
-        <row r="25">
-          <cell r="D25">
-            <v>24130054</v>
-          </cell>
-          <cell r="E25" t="str">
-            <v>رولا محمد ابراهيم نعناعه</v>
-          </cell>
-        </row>
-        <row r="26">
-          <cell r="D26">
-            <v>24130055</v>
-          </cell>
-          <cell r="E26" t="str">
-            <v>ريان احمد المهدى محمد ضيف</v>
-          </cell>
-        </row>
-        <row r="27">
-          <cell r="D27">
-            <v>24130057</v>
-          </cell>
-          <cell r="E27" t="str">
-            <v>زياد ابراهيم السيد ابراهيم السيد</v>
-          </cell>
-        </row>
-        <row r="28">
-          <cell r="D28">
-            <v>24130061</v>
-          </cell>
-          <cell r="E28" t="str">
-            <v>زينب على احمد عبد الفتاح العبد</v>
-          </cell>
-        </row>
-        <row r="29">
-          <cell r="D29">
-            <v>24130062</v>
-          </cell>
-          <cell r="E29" t="str">
-            <v>سجود عاصم ديب محمد الرباعى</v>
-          </cell>
-        </row>
-        <row r="30">
-          <cell r="D30">
-            <v>24130063</v>
-          </cell>
-          <cell r="E30" t="str">
-            <v>سلامه رجب عبد الجواد محمد راضي</v>
-          </cell>
-        </row>
-        <row r="31">
-          <cell r="D31">
-            <v>24130064</v>
-          </cell>
-          <cell r="E31" t="str">
-            <v>سما فادى ابراهيم نجيب حنين</v>
-          </cell>
-        </row>
-        <row r="32">
-          <cell r="D32">
-            <v>24130065</v>
-          </cell>
-          <cell r="E32" t="str">
-            <v>سيف الدين احمد محمود محمد محمود صالح</v>
-          </cell>
-        </row>
-        <row r="33">
-          <cell r="D33">
-            <v>24130068</v>
-          </cell>
-          <cell r="E33" t="str">
-            <v>شهد امري حامد محمد غنيم</v>
-          </cell>
-        </row>
-        <row r="34">
-          <cell r="D34">
-            <v>24130069</v>
-          </cell>
-          <cell r="E34" t="str">
-            <v>شهد رجب عادل محمد احمد</v>
-          </cell>
-        </row>
-        <row r="35">
-          <cell r="D35">
-            <v>24130080</v>
-          </cell>
-          <cell r="E35" t="str">
-            <v>عبد الله الداودى محمد رمضان السايس</v>
-          </cell>
-        </row>
-        <row r="36">
-          <cell r="D36">
-            <v>24130082</v>
-          </cell>
-          <cell r="E36" t="str">
-            <v>عبد الله محمد جابر محمد السخرى</v>
-          </cell>
-        </row>
-        <row r="37">
-          <cell r="D37">
-            <v>24130084</v>
-          </cell>
-          <cell r="E37" t="str">
-            <v>عبد الملك السيد صديق محمد</v>
-          </cell>
-        </row>
-        <row r="38">
-          <cell r="D38">
-            <v>24130085</v>
-          </cell>
-          <cell r="E38" t="str">
-            <v>عدي احمد محمود محمود ابو زيد</v>
-          </cell>
-        </row>
-        <row r="39">
-          <cell r="D39">
-            <v>24130086</v>
-          </cell>
-          <cell r="E39" t="str">
-            <v>عز الدين محمد فاروق عبد العزيز عمر</v>
-          </cell>
-        </row>
-        <row r="40">
-          <cell r="D40">
-            <v>24130089</v>
-          </cell>
-          <cell r="E40" t="str">
-            <v>علي محمد على محمد احمد عبد الله</v>
-          </cell>
-        </row>
-        <row r="41">
-          <cell r="D41">
-            <v>24130091</v>
-          </cell>
-          <cell r="E41" t="str">
-            <v>عمر محمد سعد محمد خلف</v>
-          </cell>
-        </row>
-        <row r="42">
-          <cell r="D42">
-            <v>24130096</v>
-          </cell>
-          <cell r="E42" t="str">
-            <v>فارس محمد ابراهيم احمد ابراهيم الكحكى</v>
-          </cell>
-        </row>
-        <row r="43">
-          <cell r="D43">
-            <v>24130102</v>
-          </cell>
-          <cell r="E43" t="str">
-            <v>لوجينا محمد حسين احمد على</v>
-          </cell>
-        </row>
-        <row r="44">
-          <cell r="D44">
-            <v>24130105</v>
-          </cell>
-          <cell r="E44" t="str">
-            <v>مجدي اشرف عبدالمنعم محمد على البلتاجى</v>
-          </cell>
-        </row>
-        <row r="45">
-          <cell r="D45">
-            <v>24130106</v>
-          </cell>
-          <cell r="E45" t="str">
-            <v>محمد احمد احمد سليمان ضبيع</v>
-          </cell>
-        </row>
-        <row r="46">
-          <cell r="D46">
-            <v>24130112</v>
-          </cell>
-          <cell r="E46" t="str">
-            <v>محمد البدري محمود البدري ابو عكر</v>
-          </cell>
-        </row>
-        <row r="47">
-          <cell r="D47">
-            <v>24130116</v>
-          </cell>
-          <cell r="E47" t="str">
-            <v>محمد حسين محمد حسين</v>
-          </cell>
-        </row>
-        <row r="48">
-          <cell r="D48">
-            <v>24130119</v>
-          </cell>
-          <cell r="E48" t="str">
-            <v>محمد زكي عوض عبد الله السايس</v>
-          </cell>
-        </row>
-        <row r="49">
-          <cell r="D49">
-            <v>24130122</v>
-          </cell>
-          <cell r="E49" t="str">
-            <v>محمد شريف محمد شلبى</v>
-          </cell>
-        </row>
-        <row r="50">
-          <cell r="D50">
-            <v>24130128</v>
-          </cell>
-          <cell r="E50" t="str">
-            <v>محمد عزت فوزي عبد الجليل طلبه</v>
-          </cell>
-        </row>
-        <row r="51">
-          <cell r="D51">
-            <v>24130129</v>
-          </cell>
-          <cell r="E51" t="str">
-            <v>محمد على اسماعيل علي حلاوه</v>
-          </cell>
-        </row>
-        <row r="52">
-          <cell r="D52">
-            <v>24130136</v>
-          </cell>
-          <cell r="E52" t="str">
-            <v>محمد محمد على السيد حسب الله</v>
-          </cell>
-        </row>
-        <row r="53">
-          <cell r="D53">
-            <v>24130140</v>
-          </cell>
-          <cell r="E53" t="str">
-            <v>محمد وجيه نعيم عبدالمنعم تعلب</v>
-          </cell>
-        </row>
-        <row r="54">
-          <cell r="D54">
-            <v>24130141</v>
-          </cell>
-          <cell r="E54" t="str">
-            <v>محمد ياسر سيد الشاعر</v>
-          </cell>
-        </row>
-        <row r="55">
-          <cell r="D55">
-            <v>24130145</v>
-          </cell>
-          <cell r="E55" t="str">
-            <v>محمود محمد محمود احمد السيد</v>
-          </cell>
-        </row>
-        <row r="56">
-          <cell r="D56">
-            <v>24130146</v>
-          </cell>
-          <cell r="E56" t="str">
-            <v>محمود محمد محمود توفيق الطنطاوي</v>
-          </cell>
-        </row>
-        <row r="57">
-          <cell r="D57">
-            <v>24130153</v>
-          </cell>
-          <cell r="E57" t="str">
-            <v>معاذ بديع صبح عبده حجازى</v>
-          </cell>
-        </row>
-        <row r="58">
-          <cell r="D58">
-            <v>24130156</v>
-          </cell>
-          <cell r="E58" t="str">
-            <v>ملك مجدى احمد فؤاد محمد رسلان</v>
-          </cell>
-        </row>
-        <row r="59">
-          <cell r="D59">
-            <v>24130160</v>
-          </cell>
-          <cell r="E59" t="str">
-            <v>ندى محمد صبري احمد السيد</v>
-          </cell>
-        </row>
-        <row r="60">
-          <cell r="D60">
-            <v>24130161</v>
-          </cell>
-          <cell r="E60" t="str">
-            <v>نور احمد احمد ابراهيم درويش</v>
-          </cell>
-        </row>
-        <row r="61">
-          <cell r="D61">
-            <v>24130163</v>
-          </cell>
-          <cell r="E61" t="str">
-            <v>هنا وليد محمد محمد الفطايرى</v>
-          </cell>
-        </row>
-        <row r="62">
-          <cell r="D62">
-            <v>24130167</v>
-          </cell>
-          <cell r="E62" t="str">
-            <v>يوسف احمد غالب تك كوجن</v>
-          </cell>
-        </row>
-        <row r="63">
-          <cell r="D63">
-            <v>24130171</v>
-          </cell>
-          <cell r="E63" t="str">
-            <v>يوسف عزوز انيس احمد</v>
-          </cell>
-        </row>
-        <row r="64">
-          <cell r="D64">
-            <v>24130172</v>
-          </cell>
-          <cell r="E64" t="str">
-            <v>يوسف علاء سعيد محمود ابراهيم</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1371,56 +871,56 @@
     <row r="2" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="2"/>
-      <c r="C2" s="23" t="s">
+      <c r="C2" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="2"/>
-      <c r="C3" s="23" t="s">
+      <c r="C3" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
       <c r="G3" s="2"/>
     </row>
     <row r="4" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="2"/>
-      <c r="C4" s="23" t="s">
+      <c r="C4" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
       <c r="G4" s="2"/>
     </row>
     <row r="5" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="2"/>
-      <c r="C5" s="23" t="s">
+      <c r="C5" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16"/>
       <c r="G5" s="2"/>
     </row>
     <row r="6" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="2"/>
-      <c r="C6" s="24" t="s">
+      <c r="C6" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="10"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
       <c r="G6" s="2"/>
     </row>
     <row r="7" spans="1:7" ht="20" thickBot="1" x14ac:dyDescent="0.3">
@@ -1440,27 +940,26 @@
       <c r="C8" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="D8" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="E8" s="19"/>
-      <c r="F8" s="20"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="11"/>
       <c r="G8" s="3" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="21" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
-      <c r="B9" s="3" t="str">
-        <f t="array" ref="B9">IFERROR(INDEX('[1]2nd AI-Print'!$D$9:$D$64, MATCH(D8, '[1]2nd AI-Print'!$E$9:$E$64, 0)), "")</f>
-        <v/>
+      <c r="B9" s="3" t="s">
+        <v>28</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D9" s="27"/>
-      <c r="E9" s="19"/>
-      <c r="F9" s="20"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="11"/>
       <c r="G9" s="3" t="s">
         <v>9</v>
       </c>
@@ -1484,14 +983,14 @@
     </row>
     <row r="11" spans="1:7" ht="20" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
-      <c r="B11" s="28"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="20"/>
-      <c r="F11" s="29" t="s">
+      <c r="B11" s="23"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="G11" s="20"/>
+      <c r="G11" s="11"/>
     </row>
     <row r="12" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
@@ -1504,15 +1003,15 @@
     </row>
     <row r="13" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A13" s="1"/>
-      <c r="B13" s="30" t="s">
+      <c r="B13" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="17"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="30" t="s">
+      <c r="C13" s="26"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="F13" s="14"/>
+      <c r="F13" s="19"/>
       <c r="G13" s="5"/>
     </row>
     <row r="14" spans="1:7" ht="20" x14ac:dyDescent="0.2">
@@ -1520,135 +1019,135 @@
       <c r="B14" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="D14" s="14"/>
+      <c r="D14" s="19"/>
       <c r="E14" s="6" t="s">
         <v>19</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="G14" s="25"/>
+      <c r="G14" s="20"/>
     </row>
     <row r="15" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A15" s="1"/>
       <c r="B15" s="6"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="12"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="30"/>
       <c r="E15" s="6"/>
       <c r="F15" s="6"/>
-      <c r="G15" s="26"/>
+      <c r="G15" s="21"/>
     </row>
     <row r="16" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A16" s="1"/>
       <c r="B16" s="6"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="12"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="30"/>
       <c r="E16" s="6"/>
       <c r="F16" s="6"/>
-      <c r="G16" s="26"/>
+      <c r="G16" s="21"/>
     </row>
     <row r="17" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
       <c r="B17" s="6"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="12"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="30"/>
       <c r="E17" s="6"/>
       <c r="F17" s="6"/>
-      <c r="G17" s="26"/>
+      <c r="G17" s="21"/>
     </row>
     <row r="18" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A18" s="1"/>
       <c r="B18" s="6"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="12"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="30"/>
       <c r="E18" s="6"/>
       <c r="F18" s="6"/>
-      <c r="G18" s="26"/>
+      <c r="G18" s="21"/>
     </row>
     <row r="19" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A19" s="1"/>
       <c r="B19" s="6"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="12"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="30"/>
       <c r="E19" s="6"/>
       <c r="F19" s="6"/>
-      <c r="G19" s="26"/>
+      <c r="G19" s="21"/>
     </row>
     <row r="20" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>
       <c r="B20" s="6"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="12"/>
+      <c r="C20" s="18"/>
+      <c r="D20" s="30"/>
       <c r="E20" s="6"/>
       <c r="F20" s="6"/>
-      <c r="G20" s="26"/>
+      <c r="G20" s="21"/>
     </row>
     <row r="21" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A21" s="1"/>
-      <c r="B21" s="16" t="s">
+      <c r="B21" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="C21" s="21"/>
-      <c r="D21" s="21"/>
-      <c r="E21" s="21"/>
-      <c r="F21" s="21"/>
-      <c r="G21" s="22"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="13"/>
+      <c r="F21" s="13"/>
+      <c r="G21" s="14"/>
     </row>
     <row r="22" spans="1:7" ht="20" x14ac:dyDescent="0.2">
       <c r="A22" s="1"/>
       <c r="B22" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C22" s="11" t="s">
+      <c r="C22" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="D22" s="14"/>
+      <c r="D22" s="19"/>
       <c r="E22" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F22" s="11" t="s">
+      <c r="F22" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="G22" s="14"/>
+      <c r="G22" s="19"/>
     </row>
     <row r="23" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A23" s="1"/>
       <c r="B23" s="7"/>
-      <c r="C23" s="13"/>
-      <c r="D23" s="14"/>
+      <c r="C23" s="28"/>
+      <c r="D23" s="19"/>
       <c r="E23" s="6"/>
-      <c r="F23" s="15"/>
-      <c r="G23" s="14"/>
+      <c r="F23" s="27"/>
+      <c r="G23" s="19"/>
     </row>
     <row r="24" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A24" s="1"/>
       <c r="B24" s="7"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="14"/>
+      <c r="C24" s="28"/>
+      <c r="D24" s="19"/>
       <c r="E24" s="6"/>
-      <c r="F24" s="15"/>
-      <c r="G24" s="14"/>
+      <c r="F24" s="27"/>
+      <c r="G24" s="19"/>
     </row>
     <row r="25" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A25" s="1"/>
       <c r="B25" s="7"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="14"/>
+      <c r="C25" s="28"/>
+      <c r="D25" s="19"/>
       <c r="E25" s="6"/>
-      <c r="F25" s="15"/>
-      <c r="G25" s="14"/>
+      <c r="F25" s="27"/>
+      <c r="G25" s="19"/>
     </row>
     <row r="26" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A26" s="1"/>
       <c r="B26" s="7"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="14"/>
+      <c r="C26" s="28"/>
+      <c r="D26" s="19"/>
       <c r="E26" s="6"/>
-      <c r="F26" s="15"/>
-      <c r="G26" s="14"/>
+      <c r="F26" s="27"/>
+      <c r="G26" s="19"/>
     </row>
     <row r="27" spans="1:7" ht="19" x14ac:dyDescent="0.2">
       <c r="A27" s="1"/>
@@ -1656,13 +1155,13 @@
         <f>SUM(B15:B20,B23:B26)</f>
         <v>0</v>
       </c>
-      <c r="C27" s="16" t="s">
+      <c r="C27" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="D27" s="17"/>
-      <c r="E27" s="17"/>
-      <c r="F27" s="17"/>
-      <c r="G27" s="14"/>
+      <c r="D27" s="26"/>
+      <c r="E27" s="26"/>
+      <c r="F27" s="26"/>
+      <c r="G27" s="19"/>
     </row>
     <row r="28" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
@@ -1677,10 +1176,10 @@
       <c r="A29" s="1"/>
       <c r="B29" s="2"/>
       <c r="C29" s="8"/>
-      <c r="D29" s="9" t="s">
+      <c r="D29" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="E29" s="10"/>
+      <c r="E29" s="16"/>
       <c r="F29" s="2"/>
       <c r="G29" s="8" t="s">
         <v>24</v>
@@ -1690,8 +1189,8 @@
       <c r="A30" s="1"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
-      <c r="D30" s="9"/>
-      <c r="E30" s="10"/>
+      <c r="D30" s="29"/>
+      <c r="E30" s="16"/>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
     </row>
@@ -1706,10 +1205,10 @@
     </row>
     <row r="32" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
-      <c r="B32" s="9" t="s">
+      <c r="B32" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="C32" s="10"/>
+      <c r="C32" s="16"/>
       <c r="D32" s="2"/>
       <c r="E32" s="2"/>
       <c r="F32" s="2"/>
@@ -1717,10 +1216,10 @@
     </row>
     <row r="33" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
-      <c r="B33" s="9" t="s">
+      <c r="B33" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="C33" s="10"/>
+      <c r="C33" s="16"/>
       <c r="D33" s="2"/>
       <c r="E33" s="2"/>
       <c r="F33" s="2"/>
@@ -1728,6 +1227,27 @@
     </row>
   </sheetData>
   <mergeCells count="35">
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="C27:G27"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="F23:G23"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="F24:G24"/>
     <mergeCell ref="D8:F8"/>
     <mergeCell ref="B21:G21"/>
     <mergeCell ref="C2:F2"/>
@@ -1742,27 +1262,6 @@
     <mergeCell ref="F11:G11"/>
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="E13:F13"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="F26:G26"/>
-    <mergeCell ref="C27:G27"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="F23:G23"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C25:D25"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>